<commit_message>
Changes For the Date 25th Aug 2026
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5c0380aa2ae1acd0/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5c0380aa2ae1acd0/Desktop/Daily Task/12603644/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="98" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CB51A8FC-3000-45B6-948F-0E16D4EDB2EB}"/>
+  <xr:revisionPtr revIDLastSave="113" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{32F6585C-BFE5-49C6-99AC-6CA045D1E1F6}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="66">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -232,6 +232,9 @@
   </si>
   <si>
     <t>I do a bunch of Analytical  Maths .</t>
+  </si>
+  <si>
+    <t>Researching about MMDR which is newly launched by Central Govt.</t>
   </si>
 </sst>
 </file>
@@ -512,10 +515,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1293,27 +1292,51 @@
         <v>64</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A12" s="13"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="15" t="str">
+    <row r="12" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="13">
+        <v>46259</v>
+      </c>
+      <c r="B12" s="14">
+        <v>400</v>
+      </c>
+      <c r="C12" s="14">
+        <v>133</v>
+      </c>
+      <c r="D12" s="14">
+        <v>180</v>
+      </c>
+      <c r="E12" s="14">
+        <v>30</v>
+      </c>
+      <c r="F12" s="14">
+        <v>420</v>
+      </c>
+      <c r="G12" s="14">
+        <v>6</v>
+      </c>
+      <c r="H12" s="14">
+        <v>200</v>
+      </c>
+      <c r="I12" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J12" s="15" t="str">
+        <v>1363</v>
+      </c>
+      <c r="J12" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K12" s="16"/>
-      <c r="L12" s="16"/>
-      <c r="M12" s="16"/>
-      <c r="N12" s="17"/>
+        <v>77</v>
+      </c>
+      <c r="K12" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L12" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M12" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="N12" s="17" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" s="13"/>

</xml_diff>

<commit_message>
Daily log - 2026-08-29
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -1462,14 +1462,30 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="n"/>
-      <c r="B16" s="14" t="n"/>
-      <c r="C16" s="14" t="n"/>
-      <c r="D16" s="14" t="n"/>
-      <c r="E16" s="14" t="n"/>
-      <c r="F16" s="14" t="n"/>
-      <c r="G16" s="14" t="n"/>
-      <c r="H16" s="14" t="n"/>
+      <c r="A16" s="23" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B16" s="14" t="n">
+        <v>480</v>
+      </c>
+      <c r="C16" s="14" t="n">
+        <v>80</v>
+      </c>
+      <c r="D16" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E16" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F16" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="14" t="n">
+        <v>300</v>
+      </c>
       <c r="I16" s="15">
         <f>IF(SUM(B16:F16,H16)=0,"",SUM(B16:F16,H16))</f>
         <v/>
@@ -1478,10 +1494,26 @@
         <f>IF(I16="","",1440-I16)</f>
         <v/>
       </c>
-      <c r="K16" s="16" t="n"/>
-      <c r="L16" s="16" t="n"/>
-      <c r="M16" s="16" t="n"/>
-      <c r="N16" s="17" t="n"/>
+      <c r="K16" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L16" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M16" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>Not As Good as I Expected . Disappointing</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-08-30
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -1516,14 +1516,30 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="n"/>
-      <c r="B17" s="14" t="n"/>
-      <c r="C17" s="14" t="n"/>
-      <c r="D17" s="14" t="n"/>
-      <c r="E17" s="14" t="n"/>
-      <c r="F17" s="14" t="n"/>
-      <c r="G17" s="14" t="n"/>
-      <c r="H17" s="14" t="n"/>
+      <c r="A17" s="23" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B17" s="14" t="n">
+        <v>480</v>
+      </c>
+      <c r="C17" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="D17" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E17" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F17" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="14" t="n">
+        <v>350</v>
+      </c>
       <c r="I17" s="15">
         <f>IF(SUM(B17:F17,H17)=0,"",SUM(B17:F17,H17))</f>
         <v/>
@@ -1532,10 +1548,26 @@
         <f>IF(I17="","",1440-I17)</f>
         <v/>
       </c>
-      <c r="K17" s="16" t="n"/>
-      <c r="L17" s="16" t="n"/>
-      <c r="M17" s="16" t="n"/>
-      <c r="N17" s="17" t="n"/>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M17" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N17" s="17" t="inlineStr">
+        <is>
+          <t>No Comments</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-08-31
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -1570,14 +1570,30 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="n"/>
-      <c r="B18" s="14" t="n"/>
-      <c r="C18" s="14" t="n"/>
-      <c r="D18" s="14" t="n"/>
-      <c r="E18" s="14" t="n"/>
-      <c r="F18" s="14" t="n"/>
-      <c r="G18" s="14" t="n"/>
-      <c r="H18" s="14" t="n"/>
+      <c r="A18" s="23" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B18" s="14" t="n">
+        <v>480</v>
+      </c>
+      <c r="C18" s="14" t="n">
+        <v>150</v>
+      </c>
+      <c r="D18" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E18" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F18" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H18" s="14" t="n">
+        <v>250</v>
+      </c>
       <c r="I18" s="15">
         <f>IF(SUM(B18:F18,H18)=0,"",SUM(B18:F18,H18))</f>
         <v/>
@@ -1586,10 +1602,26 @@
         <f>IF(I18="","",1440-I18)</f>
         <v/>
       </c>
-      <c r="K18" s="16" t="n"/>
-      <c r="L18" s="16" t="n"/>
-      <c r="M18" s="16" t="n"/>
-      <c r="N18" s="17" t="n"/>
+      <c r="K18" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L18" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M18" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>Just Preparing For CA</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-01
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -1624,14 +1624,30 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="n"/>
-      <c r="B19" s="14" t="n"/>
-      <c r="C19" s="14" t="n"/>
-      <c r="D19" s="14" t="n"/>
-      <c r="E19" s="14" t="n"/>
-      <c r="F19" s="14" t="n"/>
-      <c r="G19" s="14" t="n"/>
-      <c r="H19" s="14" t="n"/>
+      <c r="A19" s="23" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B19" s="14" t="n">
+        <v>480</v>
+      </c>
+      <c r="C19" s="14" t="n">
+        <v>141</v>
+      </c>
+      <c r="D19" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E19" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F19" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="G19" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="H19" s="14" t="n">
+        <v>240</v>
+      </c>
       <c r="I19" s="15">
         <f>IF(SUM(B19:F19,H19)=0,"",SUM(B19:F19,H19))</f>
         <v/>
@@ -1640,10 +1656,26 @@
         <f>IF(I19="","",1440-I19)</f>
         <v/>
       </c>
-      <c r="K19" s="16" t="n"/>
-      <c r="L19" s="16" t="n"/>
-      <c r="M19" s="16" t="n"/>
-      <c r="N19" s="17" t="n"/>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M19" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N19" s="17" t="inlineStr">
+        <is>
+          <t>It's a Hectic day .</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-02
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -1678,14 +1678,30 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="n"/>
-      <c r="B20" s="14" t="n"/>
-      <c r="C20" s="14" t="n"/>
-      <c r="D20" s="14" t="n"/>
-      <c r="E20" s="14" t="n"/>
-      <c r="F20" s="14" t="n"/>
-      <c r="G20" s="14" t="n"/>
-      <c r="H20" s="14" t="n"/>
+      <c r="A20" s="23" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B20" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C20" s="14" t="n">
+        <v>150</v>
+      </c>
+      <c r="D20" s="14" t="n">
+        <v>180</v>
+      </c>
+      <c r="E20" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="G20" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="H20" s="14" t="n">
+        <v>240</v>
+      </c>
       <c r="I20" s="15">
         <f>IF(SUM(B20:F20,H20)=0,"",SUM(B20:F20,H20))</f>
         <v/>
@@ -1694,10 +1710,26 @@
         <f>IF(I20="","",1440-I20)</f>
         <v/>
       </c>
-      <c r="K20" s="16" t="n"/>
-      <c r="L20" s="16" t="n"/>
-      <c r="M20" s="16" t="n"/>
-      <c r="N20" s="17" t="n"/>
+      <c r="K20" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L20" s="16" t="inlineStr">
+        <is>
+          <t>Satisfied</t>
+        </is>
+      </c>
+      <c r="M20" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
+        <is>
+          <t>Partially Satisfied , But  I need to work on Analytical Math .</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-03
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -1732,14 +1732,30 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="n"/>
-      <c r="B21" s="14" t="n"/>
-      <c r="C21" s="14" t="n"/>
-      <c r="D21" s="14" t="n"/>
-      <c r="E21" s="14" t="n"/>
-      <c r="F21" s="14" t="n"/>
-      <c r="G21" s="14" t="n"/>
-      <c r="H21" s="14" t="n"/>
+      <c r="A21" s="23" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B21" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C21" s="14" t="n">
+        <v>151</v>
+      </c>
+      <c r="D21" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E21" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F21" s="14" t="n">
+        <v>240</v>
+      </c>
+      <c r="G21" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H21" s="14" t="n">
+        <v>300</v>
+      </c>
       <c r="I21" s="15">
         <f>IF(SUM(B21:F21,H21)=0,"",SUM(B21:F21,H21))</f>
         <v/>
@@ -1748,10 +1764,26 @@
         <f>IF(I21="","",1440-I21)</f>
         <v/>
       </c>
-      <c r="K21" s="16" t="n"/>
-      <c r="L21" s="16" t="n"/>
-      <c r="M21" s="16" t="n"/>
-      <c r="N21" s="17" t="n"/>
+      <c r="K21" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L21" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M21" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N21" s="17" t="inlineStr">
+        <is>
+          <t>I have my Communication CA today , I think i perform average on it .</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-04
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -1786,14 +1786,30 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="n"/>
-      <c r="B22" s="14" t="n"/>
-      <c r="C22" s="14" t="n"/>
-      <c r="D22" s="14" t="n"/>
-      <c r="E22" s="14" t="n"/>
-      <c r="F22" s="14" t="n"/>
-      <c r="G22" s="14" t="n"/>
-      <c r="H22" s="14" t="n"/>
+      <c r="A22" s="23" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B22" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C22" s="14" t="n">
+        <v>143</v>
+      </c>
+      <c r="D22" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E22" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F22" s="14" t="n">
+        <v>240</v>
+      </c>
+      <c r="G22" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H22" s="14" t="n">
+        <v>240</v>
+      </c>
       <c r="I22" s="15">
         <f>IF(SUM(B22:F22,H22)=0,"",SUM(B22:F22,H22))</f>
         <v/>
@@ -1802,10 +1818,26 @@
         <f>IF(I22="","",1440-I22)</f>
         <v/>
       </c>
-      <c r="K22" s="16" t="n"/>
-      <c r="L22" s="16" t="n"/>
-      <c r="M22" s="16" t="n"/>
-      <c r="N22" s="17" t="n"/>
+      <c r="K22" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L22" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M22" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N22" s="17" t="inlineStr">
+        <is>
+          <t>No comment</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-05
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -1840,14 +1840,30 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="n"/>
-      <c r="B23" s="14" t="n"/>
-      <c r="C23" s="14" t="n"/>
-      <c r="D23" s="14" t="n"/>
-      <c r="E23" s="14" t="n"/>
-      <c r="F23" s="14" t="n"/>
-      <c r="G23" s="14" t="n"/>
-      <c r="H23" s="14" t="n"/>
+      <c r="A23" s="23" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B23" s="14" t="n">
+        <v>480</v>
+      </c>
+      <c r="C23" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="D23" s="14" t="n">
+        <v>150</v>
+      </c>
+      <c r="E23" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F23" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="14" t="n">
+        <v>300</v>
+      </c>
       <c r="I23" s="15">
         <f>IF(SUM(B23:F23,H23)=0,"",SUM(B23:F23,H23))</f>
         <v/>
@@ -1856,10 +1872,26 @@
         <f>IF(I23="","",1440-I23)</f>
         <v/>
       </c>
-      <c r="K23" s="16" t="n"/>
-      <c r="L23" s="16" t="n"/>
-      <c r="M23" s="16" t="n"/>
-      <c r="N23" s="17" t="n"/>
+      <c r="K23" s="16" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="L23" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M23" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N23" s="17" t="inlineStr">
+        <is>
+          <t>Nothing special .</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-06
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -1894,14 +1894,30 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="n"/>
-      <c r="B24" s="14" t="n"/>
-      <c r="C24" s="14" t="n"/>
-      <c r="D24" s="14" t="n"/>
-      <c r="E24" s="14" t="n"/>
-      <c r="F24" s="14" t="n"/>
-      <c r="G24" s="14" t="n"/>
-      <c r="H24" s="14" t="n"/>
+      <c r="A24" s="23" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B24" s="14" t="n">
+        <v>480</v>
+      </c>
+      <c r="C24" s="14" t="n">
+        <v>126</v>
+      </c>
+      <c r="D24" s="14" t="n">
+        <v>150</v>
+      </c>
+      <c r="E24" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F24" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="14" t="n">
+        <v>300</v>
+      </c>
       <c r="I24" s="15">
         <f>IF(SUM(B24:F24,H24)=0,"",SUM(B24:F24,H24))</f>
         <v/>
@@ -1910,10 +1926,26 @@
         <f>IF(I24="","",1440-I24)</f>
         <v/>
       </c>
-      <c r="K24" s="16" t="n"/>
-      <c r="L24" s="16" t="n"/>
-      <c r="M24" s="16" t="n"/>
-      <c r="N24" s="17" t="n"/>
+      <c r="K24" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L24" s="16" t="inlineStr">
+        <is>
+          <t>Unsatisfied</t>
+        </is>
+      </c>
+      <c r="M24" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N24" s="17" t="inlineStr">
+        <is>
+          <t>I talk to  a closest freind of mine after ages .</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-07
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -1948,14 +1948,30 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="n"/>
-      <c r="B25" s="14" t="n"/>
-      <c r="C25" s="14" t="n"/>
-      <c r="D25" s="14" t="n"/>
-      <c r="E25" s="14" t="n"/>
-      <c r="F25" s="14" t="n"/>
-      <c r="G25" s="14" t="n"/>
-      <c r="H25" s="14" t="n"/>
+      <c r="A25" s="23" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B25" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C25" s="14" t="n">
+        <v>206</v>
+      </c>
+      <c r="D25" s="14" t="n">
+        <v>90</v>
+      </c>
+      <c r="E25" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F25" s="14" t="n">
+        <v>240</v>
+      </c>
+      <c r="G25" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H25" s="14" t="n">
+        <v>240</v>
+      </c>
       <c r="I25" s="15">
         <f>IF(SUM(B25:F25,H25)=0,"",SUM(B25:F25,H25))</f>
         <v/>
@@ -1964,10 +1980,26 @@
         <f>IF(I25="","",1440-I25)</f>
         <v/>
       </c>
-      <c r="K25" s="16" t="n"/>
-      <c r="L25" s="16" t="n"/>
-      <c r="M25" s="16" t="n"/>
-      <c r="N25" s="17" t="n"/>
+      <c r="K25" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L25" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M25" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N25" s="17" t="inlineStr">
+        <is>
+          <t>It's Monday .</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-08
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -2002,14 +2002,30 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="13" t="n"/>
-      <c r="B26" s="14" t="n"/>
-      <c r="C26" s="14" t="n"/>
-      <c r="D26" s="14" t="n"/>
-      <c r="E26" s="14" t="n"/>
-      <c r="F26" s="14" t="n"/>
-      <c r="G26" s="14" t="n"/>
-      <c r="H26" s="14" t="n"/>
+      <c r="A26" s="23" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B26" s="14" t="n">
+        <v>480</v>
+      </c>
+      <c r="C26" s="14" t="n">
+        <v>153</v>
+      </c>
+      <c r="D26" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E26" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="G26" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H26" s="14" t="n">
+        <v>240</v>
+      </c>
       <c r="I26" s="15">
         <f>IF(SUM(B26:F26,H26)=0,"",SUM(B26:F26,H26))</f>
         <v/>
@@ -2018,10 +2034,26 @@
         <f>IF(I26="","",1440-I26)</f>
         <v/>
       </c>
-      <c r="K26" s="16" t="n"/>
-      <c r="L26" s="16" t="n"/>
-      <c r="M26" s="16" t="n"/>
-      <c r="N26" s="17" t="n"/>
+      <c r="K26" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L26" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M26" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N26" s="17" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-09
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -2056,14 +2056,30 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="n"/>
-      <c r="B27" s="14" t="n"/>
-      <c r="C27" s="14" t="n"/>
-      <c r="D27" s="14" t="n"/>
-      <c r="E27" s="14" t="n"/>
-      <c r="F27" s="14" t="n"/>
-      <c r="G27" s="14" t="n"/>
-      <c r="H27" s="14" t="n"/>
+      <c r="A27" s="23" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B27" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C27" s="14" t="n">
+        <v>204</v>
+      </c>
+      <c r="D27" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="E27" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F27" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="G27" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H27" s="14" t="n">
+        <v>220</v>
+      </c>
       <c r="I27" s="15">
         <f>IF(SUM(B27:F27,H27)=0,"",SUM(B27:F27,H27))</f>
         <v/>
@@ -2072,10 +2088,26 @@
         <f>IF(I27="","",1440-I27)</f>
         <v/>
       </c>
-      <c r="K27" s="16" t="n"/>
-      <c r="L27" s="16" t="n"/>
-      <c r="M27" s="16" t="n"/>
-      <c r="N27" s="17" t="n"/>
+      <c r="K27" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L27" s="16" t="inlineStr">
+        <is>
+          <t>Unsatisfied</t>
+        </is>
+      </c>
+      <c r="M27" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N27" s="17" t="inlineStr">
+        <is>
+          <t>It was a bit furstrating cause im unable to match my expections .</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-10
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -2110,14 +2110,30 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="n"/>
-      <c r="B28" s="14" t="n"/>
-      <c r="C28" s="14" t="n"/>
-      <c r="D28" s="14" t="n"/>
-      <c r="E28" s="14" t="n"/>
-      <c r="F28" s="14" t="n"/>
-      <c r="G28" s="14" t="n"/>
-      <c r="H28" s="14" t="n"/>
+      <c r="A28" s="23" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B28" s="14" t="n">
+        <v>480</v>
+      </c>
+      <c r="C28" s="14" t="n">
+        <v>115</v>
+      </c>
+      <c r="D28" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="E28" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F28" s="14" t="n">
+        <v>240</v>
+      </c>
+      <c r="G28" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H28" s="14" t="n">
+        <v>220</v>
+      </c>
       <c r="I28" s="15">
         <f>IF(SUM(B28:F28,H28)=0,"",SUM(B28:F28,H28))</f>
         <v/>
@@ -2126,10 +2142,26 @@
         <f>IF(I28="","",1440-I28)</f>
         <v/>
       </c>
-      <c r="K28" s="16" t="n"/>
-      <c r="L28" s="16" t="n"/>
-      <c r="M28" s="16" t="n"/>
-      <c r="N28" s="17" t="n"/>
+      <c r="K28" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L28" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M28" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N28" s="17" t="inlineStr">
+        <is>
+          <t>It was Freshers Party today .</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="13" t="n"/>

</xml_diff>

<commit_message>
Daily log - 2026-09-11
</commit_message>
<xml_diff>
--- a/12603644.xlsx
+++ b/12603644.xlsx
@@ -2164,14 +2164,30 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="n"/>
-      <c r="B29" s="14" t="n"/>
-      <c r="C29" s="14" t="n"/>
-      <c r="D29" s="14" t="n"/>
-      <c r="E29" s="14" t="n"/>
-      <c r="F29" s="14" t="n"/>
-      <c r="G29" s="14" t="n"/>
-      <c r="H29" s="14" t="n"/>
+      <c r="A29" s="23" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B29" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="C29" s="14" t="n">
+        <v>144</v>
+      </c>
+      <c r="D29" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="E29" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="14" t="n">
+        <v>240</v>
+      </c>
+      <c r="G29" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H29" s="14" t="n">
+        <v>250</v>
+      </c>
       <c r="I29" s="15">
         <f>IF(SUM(B29:F29,H29)=0,"",SUM(B29:F29,H29))</f>
         <v/>
@@ -2180,10 +2196,26 @@
         <f>IF(I29="","",1440-I29)</f>
         <v/>
       </c>
-      <c r="K29" s="16" t="n"/>
-      <c r="L29" s="16" t="n"/>
-      <c r="M29" s="16" t="n"/>
-      <c r="N29" s="17" t="n"/>
+      <c r="K29" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L29" s="16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="M29" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N29" s="17" t="inlineStr">
+        <is>
+          <t>Seeking my acedemic comeback.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="13" t="n"/>

</xml_diff>